<commit_message>
Add new evaluation results and update README with Fine-tuned CV + Synth No Morph metrics
- Introduced new evaluation JSON files for Slovenian language under parakeetV3/sl, including test, validation, and FLEURS datasets.
- Updated README.md to include results for Fine-tuned CV + Synth No Morph configurations, reflecting the latest WER and CER metrics.
- Added a training script for fine-tuning Whisper model with specified configurations.
</commit_message>
<xml_diff>
--- a/results/normalized_results.xlsx
+++ b/results/normalized_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1278,6 +1278,120 @@
         <v>-3.64</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>parakeet-tdt-cv_synth_no_morph_sl-seed42</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>cv17_test</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1242</v>
+      </c>
+      <c r="E23" t="n">
+        <v>12.22</v>
+      </c>
+      <c r="F23" t="n">
+        <v>9.68</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-2.54</v>
+      </c>
+      <c r="H23" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="I23" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="J23" t="n">
+        <v>-0.45</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>parakeet-tdt-cv_synth_no_morph_sl-seed42</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>cv17_validation</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1232</v>
+      </c>
+      <c r="E24" t="n">
+        <v>11.62</v>
+      </c>
+      <c r="F24" t="n">
+        <v>9.210000000000001</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-2.41</v>
+      </c>
+      <c r="H24" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="I24" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="J24" t="n">
+        <v>-0.41</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>parakeet-tdt-cv_synth_no_morph_sl-seed42</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>fleurs_test</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>834</v>
+      </c>
+      <c r="E25" t="n">
+        <v>35.05</v>
+      </c>
+      <c r="F25" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="G25" t="n">
+        <v>-17.15</v>
+      </c>
+      <c r="H25" t="n">
+        <v>9.68</v>
+      </c>
+      <c r="I25" t="n">
+        <v>6.03</v>
+      </c>
+      <c r="J25" t="n">
+        <v>-3.65</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Whisper-large-v3 results to README: raw, normalized, significance
Includes all Slovenian results (zero-shot, cv_only, synth_no_morph,
synth_all) and available Estonian results. Bootstrap significance
testing confirms all CV17 improvements are significant (p<0.01).
Notable: Whisper fine-tuning degrades FLEURS performance.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/normalized_results.xlsx
+++ b/results/normalized_results.xlsx
@@ -425,56 +425,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:K48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Lang</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Test Set</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Samples</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Raw WER</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Norm WER</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>WER Diff</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Raw CER</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Norm CER</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>CER Diff</t>
         </is>
@@ -483,913 +488,2022 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>parakeet-tdt-0.6b-v3</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>et</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>cv17_test</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>2653</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>27.19</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>24.58</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>-2.61</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>6.42</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>5.85</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>-0.57</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>parakeet-tdt-0.6b-v3</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>et</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>cv17_validation</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>2653</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>26.93</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>24.7</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>-2.23</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>6.26</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>5.75</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>-0.51</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>parakeet-tdt-0.6b-v3</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>et</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>fleurs_test</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>893</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>39.14</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>18.15</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>-20.99</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>7.54</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>3.87</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>-3.67</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>parakeet-tdt-cv_only_et-seed42</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>et</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>cv17_test</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>2653</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>22.35</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>19.74</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>-2.61</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>4.9</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>4.38</v>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
         <v>-0.52</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>parakeet-tdt-cv_only_et-seed42</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>et</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>cv17_validation</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>2653</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>21.49</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>19.24</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>-2.25</v>
       </c>
-      <c r="H6" t="n">
+      <c r="I6" t="n">
         <v>4.43</v>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>3.99</v>
       </c>
-      <c r="J6" t="n">
+      <c r="K6" t="n">
         <v>-0.44</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>parakeet-tdt-cv_only_et-seed42</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>et</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>fleurs_test</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>893</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>36.6</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>14.29</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>-22.31</v>
       </c>
-      <c r="H7" t="n">
+      <c r="I7" t="n">
         <v>7.12</v>
       </c>
-      <c r="I7" t="n">
+      <c r="J7" t="n">
         <v>3.34</v>
       </c>
-      <c r="J7" t="n">
+      <c r="K7" t="n">
         <v>-3.78</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>parakeet-tdt-cv_synth_all_et-seed42</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>et</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>cv17_test</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
         <v>2653</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>21.03</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>18.51</v>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>-2.52</v>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
         <v>4.64</v>
       </c>
-      <c r="I8" t="n">
+      <c r="J8" t="n">
         <v>4.13</v>
       </c>
-      <c r="J8" t="n">
+      <c r="K8" t="n">
         <v>-0.51</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>parakeet-tdt-cv_synth_all_et-seed42</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>et</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>cv17_validation</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="E9" t="n">
         <v>2653</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>20.18</v>
       </c>
-      <c r="F9" t="n">
+      <c r="G9" t="n">
         <v>17.91</v>
       </c>
-      <c r="G9" t="n">
+      <c r="H9" t="n">
         <v>-2.27</v>
       </c>
-      <c r="H9" t="n">
+      <c r="I9" t="n">
         <v>4.21</v>
       </c>
-      <c r="I9" t="n">
+      <c r="J9" t="n">
         <v>3.78</v>
       </c>
-      <c r="J9" t="n">
+      <c r="K9" t="n">
         <v>-0.43</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>parakeet-tdt-cv_synth_all_et-seed42</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>et</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>fleurs_test</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="E10" t="n">
         <v>893</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>35.29</v>
       </c>
-      <c r="F10" t="n">
+      <c r="G10" t="n">
         <v>12.36</v>
       </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>-22.93</v>
       </c>
-      <c r="H10" t="n">
+      <c r="I10" t="n">
         <v>7.06</v>
       </c>
-      <c r="I10" t="n">
+      <c r="J10" t="n">
         <v>3.24</v>
       </c>
-      <c r="J10" t="n">
+      <c r="K10" t="n">
         <v>-3.82</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>parakeet-tdt-cv_synth_no_morph_et-seed42</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>et</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>cv17_test</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="n">
         <v>2653</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>21.24</v>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>18.69</v>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>-2.55</v>
       </c>
-      <c r="H11" t="n">
+      <c r="I11" t="n">
         <v>4.73</v>
       </c>
-      <c r="I11" t="n">
+      <c r="J11" t="n">
         <v>4.22</v>
       </c>
-      <c r="J11" t="n">
+      <c r="K11" t="n">
         <v>-0.51</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>parakeet-tdt-cv_synth_no_morph_et-seed42</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>et</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>cv17_validation</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="E12" t="n">
         <v>2653</v>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>20.51</v>
       </c>
-      <c r="F12" t="n">
+      <c r="G12" t="n">
         <v>18.29</v>
       </c>
-      <c r="G12" t="n">
+      <c r="H12" t="n">
         <v>-2.22</v>
       </c>
-      <c r="H12" t="n">
+      <c r="I12" t="n">
         <v>4.29</v>
       </c>
-      <c r="I12" t="n">
+      <c r="J12" t="n">
         <v>3.85</v>
       </c>
-      <c r="J12" t="n">
+      <c r="K12" t="n">
         <v>-0.44</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>parakeet-tdt-cv_synth_no_morph_et-seed42</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>et</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>fleurs_test</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="E13" t="n">
         <v>893</v>
       </c>
-      <c r="E13" t="n">
+      <c r="F13" t="n">
         <v>35.41</v>
       </c>
-      <c r="F13" t="n">
+      <c r="G13" t="n">
         <v>12.7</v>
       </c>
-      <c r="G13" t="n">
+      <c r="H13" t="n">
         <v>-22.71</v>
       </c>
-      <c r="H13" t="n">
+      <c r="I13" t="n">
         <v>7.1</v>
       </c>
-      <c r="I13" t="n">
+      <c r="J13" t="n">
         <v>3.26</v>
       </c>
-      <c r="J13" t="n">
+      <c r="K13" t="n">
         <v>-3.84</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>parakeet-tdt-0.6b-v3</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>sl</t>
-        </is>
-      </c>
       <c r="C14" t="inlineStr">
         <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
           <t>cv17_test</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="E14" t="n">
         <v>1242</v>
       </c>
-      <c r="E14" t="n">
+      <c r="F14" t="n">
         <v>50.23</v>
       </c>
-      <c r="F14" t="n">
+      <c r="G14" t="n">
         <v>48.13</v>
       </c>
-      <c r="G14" t="n">
+      <c r="H14" t="n">
         <v>-2.1</v>
       </c>
-      <c r="H14" t="n">
+      <c r="I14" t="n">
         <v>24.51</v>
       </c>
-      <c r="I14" t="n">
+      <c r="J14" t="n">
         <v>24.42</v>
       </c>
-      <c r="J14" t="n">
+      <c r="K14" t="n">
         <v>-0.09</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
           <t>parakeet-tdt-0.6b-v3</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>sl</t>
-        </is>
-      </c>
       <c r="C15" t="inlineStr">
         <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
           <t>cv17_validation</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="E15" t="n">
         <v>1232</v>
       </c>
-      <c r="E15" t="n">
+      <c r="F15" t="n">
         <v>58.78</v>
       </c>
-      <c r="F15" t="n">
+      <c r="G15" t="n">
         <v>57.11</v>
       </c>
-      <c r="G15" t="n">
+      <c r="H15" t="n">
         <v>-1.67</v>
       </c>
-      <c r="H15" t="n">
+      <c r="I15" t="n">
         <v>31.16</v>
       </c>
-      <c r="I15" t="n">
+      <c r="J15" t="n">
         <v>31.21</v>
       </c>
-      <c r="J15" t="n">
+      <c r="K15" t="n">
         <v>0.05</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
           <t>parakeet-tdt-0.6b-v3</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>sl</t>
-        </is>
-      </c>
       <c r="C16" t="inlineStr">
         <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
           <t>fleurs_test</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="E16" t="n">
         <v>834</v>
       </c>
-      <c r="E16" t="n">
+      <c r="F16" t="n">
         <v>40.18</v>
       </c>
-      <c r="F16" t="n">
+      <c r="G16" t="n">
         <v>24.27</v>
       </c>
-      <c r="G16" t="n">
+      <c r="H16" t="n">
         <v>-15.91</v>
       </c>
-      <c r="H16" t="n">
+      <c r="I16" t="n">
         <v>11.53</v>
       </c>
-      <c r="I16" t="n">
+      <c r="J16" t="n">
         <v>7.95</v>
       </c>
-      <c r="J16" t="n">
+      <c r="K16" t="n">
         <v>-3.58</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>parakeet-tdt-cv_only_sl-seed42</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>sl</t>
-        </is>
-      </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
           <t>cv17_test</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="E17" t="n">
         <v>1242</v>
       </c>
-      <c r="E17" t="n">
+      <c r="F17" t="n">
         <v>14.08</v>
       </c>
-      <c r="F17" t="n">
+      <c r="G17" t="n">
         <v>11.69</v>
       </c>
-      <c r="G17" t="n">
+      <c r="H17" t="n">
         <v>-2.39</v>
       </c>
-      <c r="H17" t="n">
+      <c r="I17" t="n">
         <v>3.45</v>
       </c>
-      <c r="I17" t="n">
+      <c r="J17" t="n">
         <v>3.07</v>
       </c>
-      <c r="J17" t="n">
+      <c r="K17" t="n">
         <v>-0.38</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>parakeet-tdt-cv_only_sl-seed42</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>sl</t>
-        </is>
-      </c>
       <c r="C18" t="inlineStr">
         <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
           <t>cv17_validation</t>
         </is>
       </c>
-      <c r="D18" t="n">
+      <c r="E18" t="n">
         <v>1232</v>
       </c>
-      <c r="E18" t="n">
+      <c r="F18" t="n">
         <v>13.75</v>
       </c>
-      <c r="F18" t="n">
+      <c r="G18" t="n">
         <v>11.63</v>
       </c>
-      <c r="G18" t="n">
+      <c r="H18" t="n">
         <v>-2.12</v>
       </c>
-      <c r="H18" t="n">
+      <c r="I18" t="n">
         <v>3.25</v>
       </c>
-      <c r="I18" t="n">
+      <c r="J18" t="n">
         <v>2.9</v>
       </c>
-      <c r="J18" t="n">
+      <c r="K18" t="n">
         <v>-0.35</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
           <t>parakeet-tdt-cv_only_sl-seed42</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>sl</t>
-        </is>
-      </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
           <t>fleurs_test</t>
         </is>
       </c>
-      <c r="D19" t="n">
+      <c r="E19" t="n">
         <v>834</v>
       </c>
-      <c r="E19" t="n">
+      <c r="F19" t="n">
         <v>38.57</v>
       </c>
-      <c r="F19" t="n">
+      <c r="G19" t="n">
         <v>22.36</v>
       </c>
-      <c r="G19" t="n">
+      <c r="H19" t="n">
         <v>-16.21</v>
       </c>
-      <c r="H19" t="n">
+      <c r="I19" t="n">
         <v>10.3</v>
       </c>
-      <c r="I19" t="n">
+      <c r="J19" t="n">
         <v>6.7</v>
       </c>
-      <c r="J19" t="n">
+      <c r="K19" t="n">
         <v>-3.6</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
           <t>parakeet-tdt-cv_synth_all_sl-seed42</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>sl</t>
-        </is>
-      </c>
       <c r="C20" t="inlineStr">
         <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
           <t>cv17_test</t>
         </is>
       </c>
-      <c r="D20" t="n">
+      <c r="E20" t="n">
         <v>1242</v>
       </c>
-      <c r="E20" t="n">
+      <c r="F20" t="n">
         <v>11.56</v>
       </c>
-      <c r="F20" t="n">
+      <c r="G20" t="n">
         <v>9.050000000000001</v>
       </c>
-      <c r="G20" t="n">
+      <c r="H20" t="n">
         <v>-2.51</v>
       </c>
-      <c r="H20" t="n">
+      <c r="I20" t="n">
         <v>2.87</v>
       </c>
-      <c r="I20" t="n">
+      <c r="J20" t="n">
         <v>2.45</v>
       </c>
-      <c r="J20" t="n">
+      <c r="K20" t="n">
         <v>-0.42</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>parakeet-tdt-cv_synth_all_sl-seed42</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>sl</t>
-        </is>
-      </c>
       <c r="C21" t="inlineStr">
         <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
           <t>cv17_validation</t>
         </is>
       </c>
-      <c r="D21" t="n">
+      <c r="E21" t="n">
         <v>1232</v>
       </c>
-      <c r="E21" t="n">
+      <c r="F21" t="n">
         <v>11.3</v>
       </c>
-      <c r="F21" t="n">
+      <c r="G21" t="n">
         <v>8.869999999999999</v>
       </c>
-      <c r="G21" t="n">
+      <c r="H21" t="n">
         <v>-2.43</v>
       </c>
-      <c r="H21" t="n">
+      <c r="I21" t="n">
         <v>2.61</v>
       </c>
-      <c r="I21" t="n">
+      <c r="J21" t="n">
         <v>2.19</v>
       </c>
-      <c r="J21" t="n">
+      <c r="K21" t="n">
         <v>-0.42</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
           <t>parakeet-tdt-cv_synth_all_sl-seed42</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>sl</t>
-        </is>
-      </c>
       <c r="C22" t="inlineStr">
         <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
           <t>fleurs_test</t>
         </is>
       </c>
-      <c r="D22" t="n">
+      <c r="E22" t="n">
         <v>834</v>
       </c>
-      <c r="E22" t="n">
+      <c r="F22" t="n">
         <v>34.71</v>
       </c>
-      <c r="F22" t="n">
+      <c r="G22" t="n">
         <v>17.64</v>
       </c>
-      <c r="G22" t="n">
+      <c r="H22" t="n">
         <v>-17.07</v>
       </c>
-      <c r="H22" t="n">
+      <c r="I22" t="n">
         <v>9.75</v>
       </c>
-      <c r="I22" t="n">
+      <c r="J22" t="n">
         <v>6.11</v>
       </c>
-      <c r="J22" t="n">
+      <c r="K22" t="n">
         <v>-3.64</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
           <t>parakeet-tdt-cv_synth_no_morph_sl-seed42</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>sl</t>
-        </is>
-      </c>
       <c r="C23" t="inlineStr">
         <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
           <t>cv17_test</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="E23" t="n">
         <v>1242</v>
       </c>
-      <c r="E23" t="n">
+      <c r="F23" t="n">
         <v>12.22</v>
       </c>
-      <c r="F23" t="n">
+      <c r="G23" t="n">
         <v>9.68</v>
       </c>
-      <c r="G23" t="n">
+      <c r="H23" t="n">
         <v>-2.54</v>
       </c>
-      <c r="H23" t="n">
+      <c r="I23" t="n">
         <v>2.93</v>
       </c>
-      <c r="I23" t="n">
+      <c r="J23" t="n">
         <v>2.48</v>
       </c>
-      <c r="J23" t="n">
+      <c r="K23" t="n">
         <v>-0.45</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
           <t>parakeet-tdt-cv_synth_no_morph_sl-seed42</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>sl</t>
-        </is>
-      </c>
       <c r="C24" t="inlineStr">
         <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
           <t>cv17_validation</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="E24" t="n">
         <v>1232</v>
       </c>
-      <c r="E24" t="n">
+      <c r="F24" t="n">
         <v>11.62</v>
       </c>
-      <c r="F24" t="n">
+      <c r="G24" t="n">
         <v>9.210000000000001</v>
       </c>
-      <c r="G24" t="n">
+      <c r="H24" t="n">
         <v>-2.41</v>
       </c>
-      <c r="H24" t="n">
+      <c r="I24" t="n">
         <v>2.64</v>
       </c>
-      <c r="I24" t="n">
+      <c r="J24" t="n">
         <v>2.23</v>
       </c>
-      <c r="J24" t="n">
+      <c r="K24" t="n">
         <v>-0.41</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>Parakeet</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>parakeet-tdt-cv_synth_no_morph_sl-seed42</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>sl</t>
-        </is>
-      </c>
       <c r="C25" t="inlineStr">
         <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
           <t>fleurs_test</t>
         </is>
       </c>
-      <c r="D25" t="n">
+      <c r="E25" t="n">
         <v>834</v>
       </c>
-      <c r="E25" t="n">
+      <c r="F25" t="n">
         <v>35.05</v>
       </c>
-      <c r="F25" t="n">
+      <c r="G25" t="n">
         <v>17.9</v>
       </c>
-      <c r="G25" t="n">
+      <c r="H25" t="n">
         <v>-17.15</v>
       </c>
-      <c r="H25" t="n">
+      <c r="I25" t="n">
         <v>9.68</v>
       </c>
-      <c r="I25" t="n">
+      <c r="J25" t="n">
         <v>6.03</v>
       </c>
-      <c r="J25" t="n">
+      <c r="K25" t="n">
         <v>-3.65</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>whisper-large-v3</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>et</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>cv17_test</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>2653</v>
+      </c>
+      <c r="F26" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="G26" t="n">
+        <v>31.52</v>
+      </c>
+      <c r="H26" t="n">
+        <v>-2.88</v>
+      </c>
+      <c r="I26" t="n">
+        <v>8.279999999999999</v>
+      </c>
+      <c r="J26" t="n">
+        <v>7.59</v>
+      </c>
+      <c r="K26" t="n">
+        <v>-0.6899999999999999</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>whisper-large-v3</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>et</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>cv17_validation</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>2653</v>
+      </c>
+      <c r="F27" t="n">
+        <v>33.18</v>
+      </c>
+      <c r="G27" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="H27" t="n">
+        <v>-2.38</v>
+      </c>
+      <c r="I27" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="J27" t="n">
+        <v>6.81</v>
+      </c>
+      <c r="K27" t="n">
+        <v>-0.59</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>whisper-large-v3-cv_synth_all_et-seed42</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>et</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>cv17_test</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>2653</v>
+      </c>
+      <c r="F28" t="n">
+        <v>26.46</v>
+      </c>
+      <c r="G28" t="n">
+        <v>24</v>
+      </c>
+      <c r="H28" t="n">
+        <v>-2.46</v>
+      </c>
+      <c r="I28" t="n">
+        <v>6.24</v>
+      </c>
+      <c r="J28" t="n">
+        <v>5.69</v>
+      </c>
+      <c r="K28" t="n">
+        <v>-0.55</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>whisper-large-v3-cv_synth_all_et-seed42</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>et</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>cv17_validation</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>2653</v>
+      </c>
+      <c r="F29" t="n">
+        <v>25.25</v>
+      </c>
+      <c r="G29" t="n">
+        <v>23.11</v>
+      </c>
+      <c r="H29" t="n">
+        <v>-2.14</v>
+      </c>
+      <c r="I29" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="J29" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="K29" t="n">
+        <v>-0.48</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>whisper-large-v3-cv_synth_no_morph_et-seed42</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>et</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>cv17_test</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>2653</v>
+      </c>
+      <c r="F30" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="G30" t="n">
+        <v>24.01</v>
+      </c>
+      <c r="H30" t="n">
+        <v>-2.49</v>
+      </c>
+      <c r="I30" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="J30" t="n">
+        <v>5.64</v>
+      </c>
+      <c r="K30" t="n">
+        <v>-0.5600000000000001</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>whisper-large-v3-cv_synth_no_morph_et-seed42</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>et</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>cv17_validation</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>2653</v>
+      </c>
+      <c r="F31" t="n">
+        <v>25.87</v>
+      </c>
+      <c r="G31" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="H31" t="n">
+        <v>-2.17</v>
+      </c>
+      <c r="I31" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="J31" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="K31" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>whisper-large-v3-cv_synth_unfiltered_et-seed42</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>et</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>cv17_test</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>2653</v>
+      </c>
+      <c r="F32" t="n">
+        <v>27.04</v>
+      </c>
+      <c r="G32" t="n">
+        <v>24.49</v>
+      </c>
+      <c r="H32" t="n">
+        <v>-2.55</v>
+      </c>
+      <c r="I32" t="n">
+        <v>6.27</v>
+      </c>
+      <c r="J32" t="n">
+        <v>5.67</v>
+      </c>
+      <c r="K32" t="n">
+        <v>-0.6</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>whisper-large-v3-cv_synth_unfiltered_et-seed42</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>et</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>cv17_validation</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>2653</v>
+      </c>
+      <c r="F33" t="n">
+        <v>25.94</v>
+      </c>
+      <c r="G33" t="n">
+        <v>23.81</v>
+      </c>
+      <c r="H33" t="n">
+        <v>-2.13</v>
+      </c>
+      <c r="I33" t="n">
+        <v>5.65</v>
+      </c>
+      <c r="J33" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="K33" t="n">
+        <v>-0.47</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>whisper-large-v3</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>cv17_test</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>1242</v>
+      </c>
+      <c r="F34" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="G34" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="H34" t="n">
+        <v>-2.6</v>
+      </c>
+      <c r="I34" t="n">
+        <v>5.59</v>
+      </c>
+      <c r="J34" t="n">
+        <v>5.03</v>
+      </c>
+      <c r="K34" t="n">
+        <v>-0.5600000000000001</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>whisper-large-v3</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>cv17_validation</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>1232</v>
+      </c>
+      <c r="F35" t="n">
+        <v>21.36</v>
+      </c>
+      <c r="G35" t="n">
+        <v>18.45</v>
+      </c>
+      <c r="H35" t="n">
+        <v>-2.91</v>
+      </c>
+      <c r="I35" t="n">
+        <v>5.46</v>
+      </c>
+      <c r="J35" t="n">
+        <v>4.77</v>
+      </c>
+      <c r="K35" t="n">
+        <v>-0.6899999999999999</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>whisper-large-v3</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>fleurs_test</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>834</v>
+      </c>
+      <c r="F36" t="n">
+        <v>37.02</v>
+      </c>
+      <c r="G36" t="n">
+        <v>19.18</v>
+      </c>
+      <c r="H36" t="n">
+        <v>-17.84</v>
+      </c>
+      <c r="I36" t="n">
+        <v>9.369999999999999</v>
+      </c>
+      <c r="J36" t="n">
+        <v>5.45</v>
+      </c>
+      <c r="K36" t="n">
+        <v>-3.92</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>whisper-large-v3-cv_only_sl-seed42</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>cv17_test</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>1242</v>
+      </c>
+      <c r="F37" t="n">
+        <v>19.31</v>
+      </c>
+      <c r="G37" t="n">
+        <v>16.85</v>
+      </c>
+      <c r="H37" t="n">
+        <v>-2.46</v>
+      </c>
+      <c r="I37" t="n">
+        <v>4.61</v>
+      </c>
+      <c r="J37" t="n">
+        <v>4.21</v>
+      </c>
+      <c r="K37" t="n">
+        <v>-0.4</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>whisper-large-v3-cv_only_sl-seed42</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>cv17_validation</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>1232</v>
+      </c>
+      <c r="F38" t="n">
+        <v>19.87</v>
+      </c>
+      <c r="G38" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="H38" t="n">
+        <v>-2.17</v>
+      </c>
+      <c r="I38" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="J38" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="K38" t="n">
+        <v>-0.41</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>whisper-large-v3-cv_only_sl-seed42</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>fleurs_test</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>834</v>
+      </c>
+      <c r="F39" t="n">
+        <v>46.79</v>
+      </c>
+      <c r="G39" t="n">
+        <v>32.52</v>
+      </c>
+      <c r="H39" t="n">
+        <v>-14.27</v>
+      </c>
+      <c r="I39" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="J39" t="n">
+        <v>10.93</v>
+      </c>
+      <c r="K39" t="n">
+        <v>-3.57</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>whisper-large-v3-cv_synth_all_sl-seed42</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>cv17_test</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>1242</v>
+      </c>
+      <c r="F40" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="G40" t="n">
+        <v>14</v>
+      </c>
+      <c r="H40" t="n">
+        <v>-2.4</v>
+      </c>
+      <c r="I40" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="J40" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="K40" t="n">
+        <v>-0.41</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>whisper-large-v3-cv_synth_all_sl-seed42</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>cv17_validation</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>1232</v>
+      </c>
+      <c r="F41" t="n">
+        <v>15.31</v>
+      </c>
+      <c r="G41" t="n">
+        <v>13.02</v>
+      </c>
+      <c r="H41" t="n">
+        <v>-2.29</v>
+      </c>
+      <c r="I41" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="J41" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="K41" t="n">
+        <v>-0.4</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>whisper-large-v3-cv_synth_all_sl-seed42</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>fleurs_test</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>834</v>
+      </c>
+      <c r="F42" t="n">
+        <v>41.11</v>
+      </c>
+      <c r="G42" t="n">
+        <v>25.12</v>
+      </c>
+      <c r="H42" t="n">
+        <v>-15.99</v>
+      </c>
+      <c r="I42" t="n">
+        <v>11.77</v>
+      </c>
+      <c r="J42" t="n">
+        <v>8.050000000000001</v>
+      </c>
+      <c r="K42" t="n">
+        <v>-3.72</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>whisper-large-v3-cv_synth_no_morph_sl-seed42</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>cv17_test</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>1242</v>
+      </c>
+      <c r="F43" t="n">
+        <v>15.65</v>
+      </c>
+      <c r="G43" t="n">
+        <v>13.24</v>
+      </c>
+      <c r="H43" t="n">
+        <v>-2.41</v>
+      </c>
+      <c r="I43" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="J43" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="K43" t="n">
+        <v>-0.4</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>whisper-large-v3-cv_synth_no_morph_sl-seed42</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>cv17_validation</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>1232</v>
+      </c>
+      <c r="F44" t="n">
+        <v>15.08</v>
+      </c>
+      <c r="G44" t="n">
+        <v>12.98</v>
+      </c>
+      <c r="H44" t="n">
+        <v>-2.1</v>
+      </c>
+      <c r="I44" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="J44" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="K44" t="n">
+        <v>-0.36</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>whisper-large-v3-cv_synth_no_morph_sl-seed42</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>fleurs_test</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>834</v>
+      </c>
+      <c r="F45" t="n">
+        <v>40.46</v>
+      </c>
+      <c r="G45" t="n">
+        <v>24.52</v>
+      </c>
+      <c r="H45" t="n">
+        <v>-15.94</v>
+      </c>
+      <c r="I45" t="n">
+        <v>11.98</v>
+      </c>
+      <c r="J45" t="n">
+        <v>8.32</v>
+      </c>
+      <c r="K45" t="n">
+        <v>-3.66</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>whisper-large-v3-cv_synth_unfiltered_sl-seed42</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>cv17_test</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>1242</v>
+      </c>
+      <c r="F46" t="n">
+        <v>15.44</v>
+      </c>
+      <c r="G46" t="n">
+        <v>13.16</v>
+      </c>
+      <c r="H46" t="n">
+        <v>-2.28</v>
+      </c>
+      <c r="I46" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="J46" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="K46" t="n">
+        <v>-0.37</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>whisper-large-v3-cv_synth_unfiltered_sl-seed42</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>cv17_validation</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>1232</v>
+      </c>
+      <c r="F47" t="n">
+        <v>15.65</v>
+      </c>
+      <c r="G47" t="n">
+        <v>13.46</v>
+      </c>
+      <c r="H47" t="n">
+        <v>-2.19</v>
+      </c>
+      <c r="I47" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="J47" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="K47" t="n">
+        <v>-0.37</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>whisper-large-v3-cv_synth_unfiltered_sl-seed42</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>sl</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>fleurs_test</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>834</v>
+      </c>
+      <c r="F48" t="n">
+        <v>41.06</v>
+      </c>
+      <c r="G48" t="n">
+        <v>24.66</v>
+      </c>
+      <c r="H48" t="n">
+        <v>-16.4</v>
+      </c>
+      <c r="I48" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="J48" t="n">
+        <v>8.69</v>
+      </c>
+      <c r="K48" t="n">
+        <v>-3.78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Whisper evaluation results, normalized WER significance tests, and updated README
- Add all Whisper-large-v3 evaluation JSONs for Estonian and Slovenian (cv17_val, cv17_test, fleurs_test)
- Add paired bootstrap significance scripts for raw and normalized WER
- Update README with complete Whisper significance tables (raw + normalized)
- Update normalized_results.xlsx with Architecture column
- Update report_normalized.py to include Architecture field

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/normalized_results.xlsx
+++ b/results/normalized_results.xlsx
@@ -488,7 +488,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -531,7 +531,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -574,7 +574,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -660,7 +660,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -703,7 +703,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -746,7 +746,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -789,7 +789,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -832,7 +832,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -875,7 +875,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -918,7 +918,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -961,7 +961,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1004,17 +1004,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Whisper-large-v3</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>parakeet-tdt-0.6b-v3</t>
+          <t>whisper-large-v3</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>sl</t>
+          <t>et</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1023,41 +1023,41 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>1242</v>
+        <v>2653</v>
       </c>
       <c r="F14" t="n">
-        <v>50.23</v>
+        <v>34.4</v>
       </c>
       <c r="G14" t="n">
-        <v>48.13</v>
+        <v>31.52</v>
       </c>
       <c r="H14" t="n">
-        <v>-2.1</v>
+        <v>-2.88</v>
       </c>
       <c r="I14" t="n">
-        <v>24.51</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="J14" t="n">
-        <v>24.42</v>
+        <v>7.59</v>
       </c>
       <c r="K14" t="n">
-        <v>-0.09</v>
+        <v>-0.6899999999999999</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Whisper-large-v3</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>parakeet-tdt-0.6b-v3</t>
+          <t>whisper-large-v3</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>sl</t>
+          <t>et</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1066,213 +1066,213 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>1232</v>
+        <v>2653</v>
       </c>
       <c r="F15" t="n">
-        <v>58.78</v>
+        <v>33.18</v>
       </c>
       <c r="G15" t="n">
-        <v>57.11</v>
+        <v>30.8</v>
       </c>
       <c r="H15" t="n">
-        <v>-1.67</v>
+        <v>-2.38</v>
       </c>
       <c r="I15" t="n">
-        <v>31.16</v>
+        <v>7.4</v>
       </c>
       <c r="J15" t="n">
-        <v>31.21</v>
+        <v>6.81</v>
       </c>
       <c r="K15" t="n">
-        <v>0.05</v>
+        <v>-0.59</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Whisper-large-v3</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>parakeet-tdt-0.6b-v3</t>
+          <t>whisper-large-v3-cv_synth_all_et-seed42</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>sl</t>
+          <t>et</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>fleurs_test</t>
+          <t>cv17_test</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>834</v>
+        <v>2653</v>
       </c>
       <c r="F16" t="n">
-        <v>40.18</v>
+        <v>26.46</v>
       </c>
       <c r="G16" t="n">
-        <v>24.27</v>
+        <v>24</v>
       </c>
       <c r="H16" t="n">
-        <v>-15.91</v>
+        <v>-2.46</v>
       </c>
       <c r="I16" t="n">
-        <v>11.53</v>
+        <v>6.24</v>
       </c>
       <c r="J16" t="n">
-        <v>7.95</v>
+        <v>5.69</v>
       </c>
       <c r="K16" t="n">
-        <v>-3.58</v>
+        <v>-0.55</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Whisper-large-v3</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>parakeet-tdt-cv_only_sl-seed42</t>
+          <t>whisper-large-v3-cv_synth_all_et-seed42</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>sl</t>
+          <t>et</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>cv17_test</t>
+          <t>cv17_validation</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>1242</v>
+        <v>2653</v>
       </c>
       <c r="F17" t="n">
-        <v>14.08</v>
+        <v>25.25</v>
       </c>
       <c r="G17" t="n">
-        <v>11.69</v>
+        <v>23.11</v>
       </c>
       <c r="H17" t="n">
-        <v>-2.39</v>
+        <v>-2.14</v>
       </c>
       <c r="I17" t="n">
-        <v>3.45</v>
+        <v>5.63</v>
       </c>
       <c r="J17" t="n">
-        <v>3.07</v>
+        <v>5.15</v>
       </c>
       <c r="K17" t="n">
-        <v>-0.38</v>
+        <v>-0.48</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Whisper-large-v3</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>parakeet-tdt-cv_only_sl-seed42</t>
+          <t>whisper-large-v3-cv_synth_no_morph_et-seed42</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>sl</t>
+          <t>et</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>cv17_validation</t>
+          <t>cv17_test</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>1232</v>
+        <v>2653</v>
       </c>
       <c r="F18" t="n">
-        <v>13.75</v>
+        <v>26.5</v>
       </c>
       <c r="G18" t="n">
-        <v>11.63</v>
+        <v>24.01</v>
       </c>
       <c r="H18" t="n">
-        <v>-2.12</v>
+        <v>-2.49</v>
       </c>
       <c r="I18" t="n">
-        <v>3.25</v>
+        <v>6.2</v>
       </c>
       <c r="J18" t="n">
-        <v>2.9</v>
+        <v>5.64</v>
       </c>
       <c r="K18" t="n">
-        <v>-0.35</v>
+        <v>-0.5600000000000001</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Whisper-large-v3</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>parakeet-tdt-cv_only_sl-seed42</t>
+          <t>whisper-large-v3-cv_synth_no_morph_et-seed42</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>sl</t>
+          <t>et</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>fleurs_test</t>
+          <t>cv17_validation</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>834</v>
+        <v>2653</v>
       </c>
       <c r="F19" t="n">
-        <v>38.57</v>
+        <v>25.87</v>
       </c>
       <c r="G19" t="n">
-        <v>22.36</v>
+        <v>23.7</v>
       </c>
       <c r="H19" t="n">
-        <v>-16.21</v>
+        <v>-2.17</v>
       </c>
       <c r="I19" t="n">
-        <v>10.3</v>
+        <v>5.63</v>
       </c>
       <c r="J19" t="n">
-        <v>6.7</v>
+        <v>5.13</v>
       </c>
       <c r="K19" t="n">
-        <v>-3.6</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Whisper-large-v3</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>parakeet-tdt-cv_synth_all_sl-seed42</t>
+          <t>whisper-large-v3-cv_synth_unfiltered_et-seed42</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>sl</t>
+          <t>et</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1281,41 +1281,41 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>1242</v>
+        <v>2653</v>
       </c>
       <c r="F20" t="n">
-        <v>11.56</v>
+        <v>27.04</v>
       </c>
       <c r="G20" t="n">
-        <v>9.050000000000001</v>
+        <v>24.49</v>
       </c>
       <c r="H20" t="n">
-        <v>-2.51</v>
+        <v>-2.55</v>
       </c>
       <c r="I20" t="n">
-        <v>2.87</v>
+        <v>6.27</v>
       </c>
       <c r="J20" t="n">
-        <v>2.45</v>
+        <v>5.67</v>
       </c>
       <c r="K20" t="n">
-        <v>-0.42</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Whisper-large-v3</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>parakeet-tdt-cv_synth_all_sl-seed42</t>
+          <t>whisper-large-v3-cv_synth_unfiltered_et-seed42</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>sl</t>
+          <t>et</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1324,36 +1324,36 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>1232</v>
+        <v>2653</v>
       </c>
       <c r="F21" t="n">
-        <v>11.3</v>
+        <v>25.94</v>
       </c>
       <c r="G21" t="n">
-        <v>8.869999999999999</v>
+        <v>23.81</v>
       </c>
       <c r="H21" t="n">
-        <v>-2.43</v>
+        <v>-2.13</v>
       </c>
       <c r="I21" t="n">
-        <v>2.61</v>
+        <v>5.65</v>
       </c>
       <c r="J21" t="n">
-        <v>2.19</v>
+        <v>5.18</v>
       </c>
       <c r="K21" t="n">
-        <v>-0.42</v>
+        <v>-0.47</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>parakeet-tdt-cv_synth_all_sl-seed42</t>
+          <t>parakeet-tdt-0.6b-v3</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1363,40 +1363,40 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>fleurs_test</t>
+          <t>cv17_test</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>834</v>
+        <v>1242</v>
       </c>
       <c r="F22" t="n">
-        <v>34.71</v>
+        <v>50.23</v>
       </c>
       <c r="G22" t="n">
-        <v>17.64</v>
+        <v>48.13</v>
       </c>
       <c r="H22" t="n">
-        <v>-17.07</v>
+        <v>-2.1</v>
       </c>
       <c r="I22" t="n">
-        <v>9.75</v>
+        <v>24.51</v>
       </c>
       <c r="J22" t="n">
-        <v>6.11</v>
+        <v>24.42</v>
       </c>
       <c r="K22" t="n">
-        <v>-3.64</v>
+        <v>-0.09</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>parakeet-tdt-cv_synth_no_morph_sl-seed42</t>
+          <t>parakeet-tdt-0.6b-v3</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1406,40 +1406,40 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>cv17_test</t>
+          <t>cv17_validation</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>1242</v>
+        <v>1232</v>
       </c>
       <c r="F23" t="n">
-        <v>12.22</v>
+        <v>58.78</v>
       </c>
       <c r="G23" t="n">
-        <v>9.68</v>
+        <v>57.11</v>
       </c>
       <c r="H23" t="n">
-        <v>-2.54</v>
+        <v>-1.67</v>
       </c>
       <c r="I23" t="n">
-        <v>2.93</v>
+        <v>31.16</v>
       </c>
       <c r="J23" t="n">
-        <v>2.48</v>
+        <v>31.21</v>
       </c>
       <c r="K23" t="n">
-        <v>-0.45</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>parakeet-tdt-cv_synth_no_morph_sl-seed42</t>
+          <t>parakeet-tdt-0.6b-v3</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1449,40 +1449,40 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>cv17_validation</t>
+          <t>fleurs_test</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>1232</v>
+        <v>834</v>
       </c>
       <c r="F24" t="n">
-        <v>11.62</v>
+        <v>40.18</v>
       </c>
       <c r="G24" t="n">
-        <v>9.210000000000001</v>
+        <v>24.27</v>
       </c>
       <c r="H24" t="n">
-        <v>-2.41</v>
+        <v>-15.91</v>
       </c>
       <c r="I24" t="n">
-        <v>2.64</v>
+        <v>11.53</v>
       </c>
       <c r="J24" t="n">
-        <v>2.23</v>
+        <v>7.95</v>
       </c>
       <c r="K24" t="n">
-        <v>-0.41</v>
+        <v>-3.58</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Parakeet</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>parakeet-tdt-cv_synth_no_morph_sl-seed42</t>
+          <t>parakeet-tdt-cv_only_sl-seed42</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1492,131 +1492,131 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>fleurs_test</t>
+          <t>cv17_test</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>834</v>
+        <v>1242</v>
       </c>
       <c r="F25" t="n">
-        <v>35.05</v>
+        <v>14.08</v>
       </c>
       <c r="G25" t="n">
-        <v>17.9</v>
+        <v>11.69</v>
       </c>
       <c r="H25" t="n">
-        <v>-17.15</v>
+        <v>-2.39</v>
       </c>
       <c r="I25" t="n">
-        <v>9.68</v>
+        <v>3.45</v>
       </c>
       <c r="J25" t="n">
-        <v>6.03</v>
+        <v>3.07</v>
       </c>
       <c r="K25" t="n">
-        <v>-3.65</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Whisper</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>whisper-large-v3</t>
+          <t>parakeet-tdt-cv_only_sl-seed42</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>et</t>
+          <t>sl</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>cv17_test</t>
+          <t>cv17_validation</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>2653</v>
+        <v>1232</v>
       </c>
       <c r="F26" t="n">
-        <v>34.4</v>
+        <v>13.75</v>
       </c>
       <c r="G26" t="n">
-        <v>31.52</v>
+        <v>11.63</v>
       </c>
       <c r="H26" t="n">
-        <v>-2.88</v>
+        <v>-2.12</v>
       </c>
       <c r="I26" t="n">
-        <v>8.279999999999999</v>
+        <v>3.25</v>
       </c>
       <c r="J26" t="n">
-        <v>7.59</v>
+        <v>2.9</v>
       </c>
       <c r="K26" t="n">
-        <v>-0.6899999999999999</v>
+        <v>-0.35</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Whisper</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>whisper-large-v3</t>
+          <t>parakeet-tdt-cv_only_sl-seed42</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>et</t>
+          <t>sl</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>cv17_validation</t>
+          <t>fleurs_test</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>2653</v>
+        <v>834</v>
       </c>
       <c r="F27" t="n">
-        <v>33.18</v>
+        <v>38.57</v>
       </c>
       <c r="G27" t="n">
-        <v>30.8</v>
+        <v>22.36</v>
       </c>
       <c r="H27" t="n">
-        <v>-2.38</v>
+        <v>-16.21</v>
       </c>
       <c r="I27" t="n">
-        <v>7.4</v>
+        <v>10.3</v>
       </c>
       <c r="J27" t="n">
-        <v>6.81</v>
+        <v>6.7</v>
       </c>
       <c r="K27" t="n">
-        <v>-0.59</v>
+        <v>-3.6</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Whisper</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>whisper-large-v3-cv_synth_all_et-seed42</t>
+          <t>parakeet-tdt-cv_synth_all_sl-seed42</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>et</t>
+          <t>sl</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1625,41 +1625,41 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>2653</v>
+        <v>1242</v>
       </c>
       <c r="F28" t="n">
-        <v>26.46</v>
+        <v>11.56</v>
       </c>
       <c r="G28" t="n">
-        <v>24</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="H28" t="n">
-        <v>-2.46</v>
+        <v>-2.51</v>
       </c>
       <c r="I28" t="n">
-        <v>6.24</v>
+        <v>2.87</v>
       </c>
       <c r="J28" t="n">
-        <v>5.69</v>
+        <v>2.45</v>
       </c>
       <c r="K28" t="n">
-        <v>-0.55</v>
+        <v>-0.42</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Whisper</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>whisper-large-v3-cv_synth_all_et-seed42</t>
+          <t>parakeet-tdt-cv_synth_all_sl-seed42</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>et</t>
+          <t>sl</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1668,203 +1668,203 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>2653</v>
+        <v>1232</v>
       </c>
       <c r="F29" t="n">
-        <v>25.25</v>
+        <v>11.3</v>
       </c>
       <c r="G29" t="n">
-        <v>23.11</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="H29" t="n">
-        <v>-2.14</v>
+        <v>-2.43</v>
       </c>
       <c r="I29" t="n">
-        <v>5.63</v>
+        <v>2.61</v>
       </c>
       <c r="J29" t="n">
-        <v>5.15</v>
+        <v>2.19</v>
       </c>
       <c r="K29" t="n">
-        <v>-0.48</v>
+        <v>-0.42</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Whisper</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>whisper-large-v3-cv_synth_no_morph_et-seed42</t>
+          <t>parakeet-tdt-cv_synth_all_sl-seed42</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>et</t>
+          <t>sl</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>cv17_test</t>
+          <t>fleurs_test</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>2653</v>
+        <v>834</v>
       </c>
       <c r="F30" t="n">
-        <v>26.5</v>
+        <v>34.71</v>
       </c>
       <c r="G30" t="n">
-        <v>24.01</v>
+        <v>17.64</v>
       </c>
       <c r="H30" t="n">
-        <v>-2.49</v>
+        <v>-17.07</v>
       </c>
       <c r="I30" t="n">
-        <v>6.2</v>
+        <v>9.75</v>
       </c>
       <c r="J30" t="n">
-        <v>5.64</v>
+        <v>6.11</v>
       </c>
       <c r="K30" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-3.64</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Whisper</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>whisper-large-v3-cv_synth_no_morph_et-seed42</t>
+          <t>parakeet-tdt-cv_synth_no_morph_sl-seed42</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>et</t>
+          <t>sl</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>cv17_validation</t>
+          <t>cv17_test</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>2653</v>
+        <v>1242</v>
       </c>
       <c r="F31" t="n">
-        <v>25.87</v>
+        <v>12.22</v>
       </c>
       <c r="G31" t="n">
-        <v>23.7</v>
+        <v>9.68</v>
       </c>
       <c r="H31" t="n">
-        <v>-2.17</v>
+        <v>-2.54</v>
       </c>
       <c r="I31" t="n">
-        <v>5.63</v>
+        <v>2.93</v>
       </c>
       <c r="J31" t="n">
-        <v>5.13</v>
+        <v>2.48</v>
       </c>
       <c r="K31" t="n">
-        <v>-0.5</v>
+        <v>-0.45</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Whisper</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>whisper-large-v3-cv_synth_unfiltered_et-seed42</t>
+          <t>parakeet-tdt-cv_synth_no_morph_sl-seed42</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>et</t>
+          <t>sl</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>cv17_test</t>
+          <t>cv17_validation</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>2653</v>
+        <v>1232</v>
       </c>
       <c r="F32" t="n">
-        <v>27.04</v>
+        <v>11.62</v>
       </c>
       <c r="G32" t="n">
-        <v>24.49</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="H32" t="n">
-        <v>-2.55</v>
+        <v>-2.41</v>
       </c>
       <c r="I32" t="n">
-        <v>6.27</v>
+        <v>2.64</v>
       </c>
       <c r="J32" t="n">
-        <v>5.67</v>
+        <v>2.23</v>
       </c>
       <c r="K32" t="n">
-        <v>-0.6</v>
+        <v>-0.41</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Whisper</t>
+          <t>Parakeet-TDT-0.6B-v3</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>whisper-large-v3-cv_synth_unfiltered_et-seed42</t>
+          <t>parakeet-tdt-cv_synth_no_morph_sl-seed42</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>et</t>
+          <t>sl</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>cv17_validation</t>
+          <t>fleurs_test</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>2653</v>
+        <v>834</v>
       </c>
       <c r="F33" t="n">
-        <v>25.94</v>
+        <v>35.05</v>
       </c>
       <c r="G33" t="n">
-        <v>23.81</v>
+        <v>17.9</v>
       </c>
       <c r="H33" t="n">
-        <v>-2.13</v>
+        <v>-17.15</v>
       </c>
       <c r="I33" t="n">
-        <v>5.65</v>
+        <v>9.68</v>
       </c>
       <c r="J33" t="n">
-        <v>5.18</v>
+        <v>6.03</v>
       </c>
       <c r="K33" t="n">
-        <v>-0.47</v>
+        <v>-3.65</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Whisper</t>
+          <t>Whisper-large-v3</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Whisper</t>
+          <t>Whisper-large-v3</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1950,7 +1950,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Whisper</t>
+          <t>Whisper-large-v3</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1993,7 +1993,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Whisper</t>
+          <t>Whisper-large-v3</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2036,7 +2036,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Whisper</t>
+          <t>Whisper-large-v3</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2079,7 +2079,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Whisper</t>
+          <t>Whisper-large-v3</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2122,7 +2122,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Whisper</t>
+          <t>Whisper-large-v3</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2165,7 +2165,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Whisper</t>
+          <t>Whisper-large-v3</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2208,7 +2208,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Whisper</t>
+          <t>Whisper-large-v3</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2251,7 +2251,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Whisper</t>
+          <t>Whisper-large-v3</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2294,7 +2294,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Whisper</t>
+          <t>Whisper-large-v3</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2337,7 +2337,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Whisper</t>
+          <t>Whisper-large-v3</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2380,7 +2380,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Whisper</t>
+          <t>Whisper-large-v3</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2423,7 +2423,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Whisper</t>
+          <t>Whisper-large-v3</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2466,7 +2466,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Whisper</t>
+          <t>Whisper-large-v3</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">

</xml_diff>